<commit_message>
KIOSK save box ID Changes
</commit_message>
<xml_diff>
--- a/playwright-automation/test-data/test-data.xlsx
+++ b/playwright-automation/test-data/test-data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -555,9 +555,38 @@
         <v>Ordered RX candidates; test tries next when API does not trigger</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B6" t="str">
+        <v>stage</v>
+      </c>
+      <c r="C6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="D6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="E6" t="str">
+        <v>kiosk-preferences</v>
+      </c>
+      <c r="F6" t="str">
+        <v>default</v>
+      </c>
+      <c r="G6" t="str">
+        <v>kioskBoxId</v>
+      </c>
+      <c r="H6" t="str">
+        <v>26065</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Kiosk box id for admin preference update</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
suite full assign stock and pickup flow
</commit_message>
<xml_diff>
--- a/playwright-automation/test-data/test-data.xlsx
+++ b/playwright-automation/test-data/test-data.xlsx
@@ -397,18 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-    <col min="8" max="8" width="36.83203125" customWidth="1"/>
-    <col min="9" max="9" width="58.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -584,9 +573,96 @@
         <v>Kiosk box id for admin preference update</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B7" t="str">
+        <v>stage</v>
+      </c>
+      <c r="C7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="D7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="E7" t="str">
+        <v>kiosk-add-refill-items</v>
+      </c>
+      <c r="F7" t="str">
+        <v>default</v>
+      </c>
+      <c r="G7" t="str">
+        <v>stockCode</v>
+      </c>
+      <c r="H7" t="str">
+        <v>YSY6UA</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Stock code to load in kiosk add/refill items flow</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B8" t="str">
+        <v>stage</v>
+      </c>
+      <c r="C8" t="str">
+        <v>admin</v>
+      </c>
+      <c r="D8" t="str">
+        <v>admin</v>
+      </c>
+      <c r="E8" t="str">
+        <v>kiosk-pickup-order</v>
+      </c>
+      <c r="F8" t="str">
+        <v>default</v>
+      </c>
+      <c r="G8" t="str">
+        <v>pickupCode</v>
+      </c>
+      <c r="H8" t="str">
+        <v>46W3U5</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Pickup code for kiosk pickup order flow</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>stage</v>
+      </c>
+      <c r="C9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="D9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="E9" t="str">
+        <v>kiosk-pickup-order</v>
+      </c>
+      <c r="F9" t="str">
+        <v>default</v>
+      </c>
+      <c r="G9" t="str">
+        <v>pin</v>
+      </c>
+      <c r="H9" t="str">
+        <v>11112011</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PIN/keypad digits for kiosk pickup order flow</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>